<commit_message>
Modulo 5.3: Genera archivo Excel con duplicados, conflictos y errores de importación
</commit_message>
<xml_diff>
--- a/uploads/PACKING TEST CONFLICTO.xlsx
+++ b/uploads/PACKING TEST CONFLICTO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maverick.morales\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A93C73-CA63-4AFC-97C5-5D94322A543D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5179DEA8-BF4F-4BC9-9776-EB56CBB04371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
+    <workbookView xWindow="5055" yWindow="270" windowWidth="15375" windowHeight="7785" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
   </bookViews>
   <sheets>
     <sheet name="PL DETALLE" sheetId="1" r:id="rId1"/>
@@ -157,7 +157,7 @@
     <t>PRUEBA</t>
   </si>
   <si>
-    <t>PRUEBA 2</t>
+    <t>PRUEBA 3</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
se realiza modulo para cambio masivo de estado Pendiente a Despachado a tiendas seleccionadas
</commit_message>
<xml_diff>
--- a/uploads/PACKING TEST CONFLICTO.xlsx
+++ b/uploads/PACKING TEST CONFLICTO.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maverick.morales\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5179DEA8-BF4F-4BC9-9776-EB56CBB04371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7607E900-3ACC-4044-93BF-E9300718166A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5055" yWindow="270" windowWidth="15375" windowHeight="7785" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
   </bookViews>
   <sheets>
     <sheet name="PL DETALLE" sheetId="1" r:id="rId1"/>
     <sheet name="CONSOLIDADO" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">CONSOLIDADO!$A$2:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">CONSOLIDADO!$A$2:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PL DETALLE'!$A$2:$G$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="44">
   <si>
     <t>ENTREGA RECEPCIÓN NACIONAL</t>
   </si>
@@ -158,6 +158,21 @@
   </si>
   <si>
     <t>PRUEBA 3</t>
+  </si>
+  <si>
+    <t>RALC</t>
+  </si>
+  <si>
+    <t>RCOS</t>
+  </si>
+  <si>
+    <t>ELITE BRANDS</t>
+  </si>
+  <si>
+    <t>RCHI</t>
+  </si>
+  <si>
+    <t>LOREAL</t>
   </si>
 </sst>
 </file>
@@ -1189,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1A63DEB-9037-485B-8B18-0D7D96E77363}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
@@ -1267,86 +1282,162 @@
       <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="6"/>
+      <c r="A5" s="6">
+        <v>111111</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1111</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="6">
+        <v>1</v>
+      </c>
+      <c r="F5" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="7">
+      <c r="A6" s="6">
+        <v>222222</v>
+      </c>
+      <c r="B6" s="6">
+        <v>2222</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="6">
+        <v>2</v>
+      </c>
+      <c r="F6" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>333333</v>
+      </c>
+      <c r="B7" s="6">
+        <v>3333</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="6">
+        <v>3</v>
+      </c>
+      <c r="F7" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="11"/>
+    </row>
+    <row r="9" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="11"/>
+    </row>
+    <row r="10" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="7">
         <f>+SUM(E3:E4)</f>
         <v>16</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F11" s="7">
         <f>+SUM(F3:F4)</f>
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-    </row>
-    <row r="9" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+    </row>
+    <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="18"/>
-    </row>
-    <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="B14" s="16"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="18"/>
+    </row>
+    <row r="15" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="18"/>
-    </row>
-    <row r="11" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="B15" s="16"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
+    </row>
+    <row r="16" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B16" s="13">
         <v>46178</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="15"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:F6" xr:uid="{F1A63DEB-9037-485B-8B18-0D7D96E77363}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F6">
-      <sortCondition ref="B2:B6"/>
+  <autoFilter ref="A2:F11" xr:uid="{F1A63DEB-9037-485B-8B18-0D7D96E77363}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F11">
+      <sortCondition ref="B2:B11"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>